<commit_message>
Added values for experimental pKa and logD
</commit_message>
<xml_diff>
--- a/data/drug.xlsx
+++ b/data/drug.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="203">
   <si>
     <t>Drug</t>
   </si>
@@ -617,6 +617,9 @@
   </si>
   <si>
     <t>Fleroxacin</t>
+  </si>
+  <si>
+    <t>Fexofenadine</t>
   </si>
 </sst>
 </file>
@@ -643,12 +646,18 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="9"/>
+        <bgColor auto="1"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -661,16 +670,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -680,18 +689,21 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="bottom" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -710,6 +722,7 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
+      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffaaaaaa"/>
     </indexedColors>
   </colors>
@@ -909,17 +922,17 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -946,10 +959,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1188,12 +1201,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1470,7 +1483,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1497,10 +1510,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1742,7 +1755,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E203"/>
+  <dimension ref="A1:E204"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="5" width="8.85156" style="1" customWidth="1"/>
@@ -3576,6 +3589,15 @@
       <c r="D203" s="3"/>
       <c r="E203" s="3"/>
     </row>
+    <row r="204" ht="13.55" customHeight="1">
+      <c r="A204" t="s" s="4">
+        <v>202</v>
+      </c>
+      <c r="B204" s="3"/>
+      <c r="C204" s="3"/>
+      <c r="D204" s="3"/>
+      <c r="E204" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>